<commit_message>
Cost report: S3 costs for a 10 MB bucket (storage, backup, transfer)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Lab-Setup/AWS/aws-detailed-cost-report.xlsx
+++ b/Lab-Setup/AWS/aws-detailed-cost-report.xlsx
@@ -2279,7 +2279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2289,6 +2289,9 @@
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2636,6 +2639,21 @@
           <t>Backup vault copies of each GB</t>
         </is>
       </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>Per hour, 10 MB (USD)</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>Per month, 10 MB (USD)</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>One-time cross-region transfer, 10 MB (USD)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
@@ -2665,6 +2683,18 @@
       <c r="G20" s="59" t="n">
         <v>0</v>
       </c>
+      <c r="H20" s="58">
+        <f>I20/Rates!$B$4</f>
+        <v>3.076840753424657e-07</v>
+      </c>
+      <c r="I20" s="58">
+        <f>('Our stacks'!$C$7/Rates!$B$6)*(F20*Rates!$B$10+G20*Rates!$B$20)</f>
+        <v>0.00022460937499999998</v>
+      </c>
+      <c r="J20" s="58">
+        <f>('Our stacks'!$C$7/Rates!$B$6)*0*Rates!$B$13</f>
+        <v>0.0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
@@ -2694,6 +2724,18 @@
       <c r="G21" s="59" t="n">
         <v>0</v>
       </c>
+      <c r="H21" s="58">
+        <f>I21/Rates!$B$4</f>
+        <v>3.076840753424657e-07</v>
+      </c>
+      <c r="I21" s="58">
+        <f>('Our stacks'!$C$7/Rates!$B$6)*(F21*Rates!$B$10+G21*Rates!$B$20)</f>
+        <v>0.00022460937499999998</v>
+      </c>
+      <c r="J21" s="58">
+        <f>('Our stacks'!$C$7/Rates!$B$6)*0*Rates!$B$13</f>
+        <v>0.0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
@@ -2723,6 +2765,18 @@
       <c r="G22" s="59" t="n">
         <v>0</v>
       </c>
+      <c r="H22" s="58">
+        <f>I22/Rates!$B$4</f>
+        <v>3.076840753424657e-07</v>
+      </c>
+      <c r="I22" s="58">
+        <f>('Our stacks'!$C$7/Rates!$B$6)*(F22*Rates!$B$10+G22*Rates!$B$20)</f>
+        <v>0.00022460937499999998</v>
+      </c>
+      <c r="J22" s="58">
+        <f>('Our stacks'!$C$7/Rates!$B$6)*0*Rates!$B$13</f>
+        <v>0.0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
@@ -2752,6 +2806,18 @@
       <c r="G23" s="59" t="n">
         <v>0</v>
       </c>
+      <c r="H23" s="58">
+        <f>I23/Rates!$B$4</f>
+        <v>6.153681506849314e-07</v>
+      </c>
+      <c r="I23" s="58">
+        <f>('Our stacks'!$C$7/Rates!$B$6)*(F23*Rates!$B$10+G23*Rates!$B$20)</f>
+        <v>0.00044921874999999997</v>
+      </c>
+      <c r="J23" s="58">
+        <f>('Our stacks'!$C$7/Rates!$B$6)*1*Rates!$B$13</f>
+        <v>0.0001953125</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
@@ -2781,6 +2847,18 @@
       <c r="G24" s="59" t="n">
         <v>1</v>
       </c>
+      <c r="H24" s="58">
+        <f>I24/Rates!$B$4</f>
+        <v>9.765625e-07</v>
+      </c>
+      <c r="I24" s="58">
+        <f>('Our stacks'!$C$7/Rates!$B$6)*(F24*Rates!$B$10+G24*Rates!$B$20)</f>
+        <v>0.0007128906250000001</v>
+      </c>
+      <c r="J24" s="58">
+        <f>('Our stacks'!$C$7/Rates!$B$6)*0*Rates!$B$13</f>
+        <v>0.0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
@@ -2810,6 +2888,18 @@
       <c r="G25" s="59" t="n">
         <v>2</v>
       </c>
+      <c r="H25" s="58">
+        <f>I25/Rates!$B$4</f>
+        <v>1.6454409246575343e-06</v>
+      </c>
+      <c r="I25" s="58">
+        <f>('Our stacks'!$C$7/Rates!$B$6)*(F25*Rates!$B$10+G25*Rates!$B$20)</f>
+        <v>0.001201171875</v>
+      </c>
+      <c r="J25" s="58">
+        <f>('Our stacks'!$C$7/Rates!$B$6)*1*Rates!$B$23</f>
+        <v>0.0001953125</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
@@ -2839,6 +2929,18 @@
       <c r="G26" s="59" t="n">
         <v>0</v>
       </c>
+      <c r="H26" s="58">
+        <f>I26/Rates!$B$4</f>
+        <v>3.076840753424657e-07</v>
+      </c>
+      <c r="I26" s="58">
+        <f>('Our stacks'!$C$7/Rates!$B$6)*(F26*Rates!$B$10+G26*Rates!$B$20)</f>
+        <v>0.00022460937499999998</v>
+      </c>
+      <c r="J26" s="58">
+        <f>('Our stacks'!$C$7/Rates!$B$6)*0*Rates!$B$13</f>
+        <v>0.0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
@@ -2868,6 +2970,18 @@
       <c r="G27" s="59" t="n">
         <v>0</v>
       </c>
+      <c r="H27" s="58">
+        <f>I27/Rates!$B$4</f>
+        <v>9.230522260273973e-07</v>
+      </c>
+      <c r="I27" s="58">
+        <f>('Our stacks'!$C$7/Rates!$B$6)*(F27*Rates!$B$10+G27*Rates!$B$20)</f>
+        <v>0.0006738281250000001</v>
+      </c>
+      <c r="J27" s="58">
+        <f>('Our stacks'!$C$7/Rates!$B$6)*1*Rates!$B$13</f>
+        <v>0.0001953125</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
@@ -2897,6 +3011,18 @@
       <c r="G28" s="59" t="n">
         <v>2</v>
       </c>
+      <c r="H28" s="58">
+        <f>I28/Rates!$B$4</f>
+        <v>1.6454409246575343e-06</v>
+      </c>
+      <c r="I28" s="58">
+        <f>('Our stacks'!$C$7/Rates!$B$6)*(F28*Rates!$B$10+G28*Rates!$B$20)</f>
+        <v>0.001201171875</v>
+      </c>
+      <c r="J28" s="58">
+        <f>('Our stacks'!$C$7/Rates!$B$6)*1*Rates!$B$23</f>
+        <v>0.0001953125</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="9" t="inlineStr">
@@ -2925,6 +3051,18 @@
       </c>
       <c r="G29" s="59" t="n">
         <v>0</v>
+      </c>
+      <c r="H29" s="58">
+        <f>I29/Rates!$B$4</f>
+        <v>9.230522260273973e-07</v>
+      </c>
+      <c r="I29" s="58">
+        <f>('Our stacks'!$C$7/Rates!$B$6)*(F29*Rates!$B$10+G29*Rates!$B$20)</f>
+        <v>0.0006738281250000001</v>
+      </c>
+      <c r="J29" s="58">
+        <f>('Our stacks'!$C$7/Rates!$B$6)*1*Rates!$B$13</f>
+        <v>0.0001953125</v>
       </c>
     </row>
     <row r="30">
@@ -2948,18 +3086,30 @@
       </c>
       <c r="F30" s="53" t="n"/>
       <c r="G30" s="53" t="n"/>
+      <c r="H30" s="55">
+        <f>SUM(H20:H29)</f>
+        <v>7.959653253424657e-06</v>
+      </c>
+      <c r="I30" s="55">
+        <f>SUM(I20:I29)</f>
+        <v>0.005810546875</v>
+      </c>
+      <c r="J30" s="55">
+        <f>SUM(J20:J29)</f>
+        <v>0.0009765625</v>
+      </c>
     </row>
     <row r="31" ht="36" customHeight="1">
       <c r="A31" s="47" t="inlineStr">
         <is>
-          <t>Per month = bucket GB ('Our stacks'!C6, now 1 GB) x (S3 copies x S3 Standard rate + vault copies x AWS Backup rate). Not included: requests ($0.005 per 1,000 PUTs), the one-time $0.02/GB for CRR and cross-region backup copies, and old versions kept by versioning or Object Lock.</t>
+          <t>Per month = bucket GB ('Our stacks'!C6, now 1 GB; columns H-J use 'Our stacks'!C7, now 10 MB = 0.0098 GB) x (S3 copies x S3 Standard rate + vault copies x AWS Backup rate). Column J is the one-time $0.02/GB for the first CRR or cross-region backup copy (s3-04, s3-08 and s3-replication replicate one copy across regions; SRR has no transfer charge). Not included: requests ($0.005 per 1,000 PUTs), AWS Backup's 128 KB minimum per object, and old versions kept by versioning or Object Lock.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A31:G31"/>
-    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A31:J31"/>
+    <mergeCell ref="A2:J2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3088,7 +3238,21 @@
       <c r="O6" s="16" t="n"/>
       <c r="P6" s="17" t="n"/>
     </row>
-    <row r="7"/>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>Small S3 test data (MB)</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="n">
+        <v>10</v>
+      </c>
+      <c r="D7" s="15" t="inlineStr">
+        <is>
+          <t>A small test upload. Folder costs shows S3 costs for this size as well as for C6.</t>
+        </is>
+      </c>
+    </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>

</xml_diff>